<commit_message>
docs(bch): record the landed codec in the MAS, align paths with fub/macro, register the filelist area
All five MAS block pages now say landed with the RTL paths and the
implementation facts the RTL fixed (KES out_more_than_t and the RIBM-only
KES_ALGO posture; Chien raw root flags with the qualifier living in the
decoder core; decoder core RECHECK state, release-on-verdict corrections,
single-outstanding blocks, no erasure port while D5 stays open). GF import
and block-location paths follow the RS restructure (rtl/fub/gf, rtl/fub,
rtl/macro); kmap citations re-anchored to the shifted lines. Register the
bch area in bin/filelists.toml from its first RTL. CLAUDE.md records the
full-codec status and the DV run recipe (venv + SIM=verilator; cocotb_test
never rebuilds on RTL change).
</commit_message>
<xml_diff>
--- a/projects/components/ecc-ip/bch/docs/bch_signal_contracts.xlsx
+++ b/projects/components/ecc-ip/bch/docs/bch_signal_contracts.xlsx
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>rtl/bch_encoder_core.sv</t>
+          <t>rtl/macro/bch_encoder_core.sv</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>rtl/bch_syndrome_unit.sv</t>
+          <t>rtl/fub/bch_syndrome_unit.sv</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>rtl/bch_chien_search.sv</t>
+          <t>rtl/fub/bch_chien_search.sv</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>rtl/bch_decoder_core.sv</t>
+          <t>rtl/macro/bch_decoder_core.sv</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>rtl/bch_encoder_core.sv / rtl/bch_decoder_core.sv</t>
+          <t>rtl/macro/bch_encoder_core.sv / rtl/macro/bch_decoder_core.sv</t>
         </is>
       </c>
     </row>

</xml_diff>